<commit_message>
ainda arrumando pontos de observacao
</commit_message>
<xml_diff>
--- a/planilhas/equipment.xlsx
+++ b/planilhas/equipment.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1869" uniqueCount="1869">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="1877">
   <si>
     <t xml:space="preserve">Model Name</t>
   </si>
@@ -43,10 +43,10 @@
     <t xml:space="preserve">Vy</t>
   </si>
   <si>
-    <t xml:space="preserve">LarguraMetros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ComprimentoMetros</t>
+    <t xml:space="preserve">Vx_largura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vy_altura</t>
   </si>
   <si>
     <t xml:space="preserve">ARGO_PARNAIBAIII_V2_LD::ECHO_FOX::REATOR1</t>
@@ -5581,6 +5581,18 @@
     <t xml:space="preserve">[[-41.764294096417586, -3.123543183817039], [-41.764294096417586, NaN]]</t>
   </si>
   <si>
+    <t xml:space="preserve">ARGO_PARNAIBAIII_V2_LD::BASE::canaleta9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-41.764725924901775, -3.1229457840766752]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.764725924901775, -3.1229457840766752], [NaN, -3.1229457840766752]]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.764725924901775, -3.1229457840766752], [-41.764725924901775, NaN]]</t>
+  </si>
+  <si>
     <t xml:space="preserve">ARGO_PARNAIBAIII_V2_LD::BASE::talude1</t>
   </si>
   <si>
@@ -5620,13 +5632,25 @@
     <t xml:space="preserve">ARGO_PARNAIBAIII_V2_LD::BASE::talude4</t>
   </si>
   <si>
-    <t xml:space="preserve">[-41.7635473934309, -3.122882479648937]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[[-41.7635473934309, -3.122882479648937], [100.00089885919243, -3.122882479648937]]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[[-41.7635473934309, -3.122882479648937], [-41.7635473934309, 2.0000180869207522]]</t>
+    <t xml:space="preserve">[-41.763457429197345, -3.12288247955997]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.763457429197345, -3.12288247955997], [100.00089885919243, -3.12288247955997]]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.763457429197345, -3.12288247955997], [-41.763457429197345, 2.0000180869207522]]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARGO_PARNAIBAIII_V2_LD::BASE::talude5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[-41.76514060201819, -3.1237367607723403]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.76514060201819, -3.1237367607723403], [75.00067414439432, -3.1237367607723403]]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[[-41.76514060201819, -3.1237367607723403], [-41.76514060201819, 2.000018087029065]]</t>
   </si>
 </sst>
 </file>
@@ -5748,6 +5772,9 @@
   </sheetPr>
   <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="57.69"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -19152,10 +19179,10 @@
         <v>1853</v>
       </c>
       <c r="B463" s="2" t="n">
-        <v>-3.1223398743864</v>
+        <v>-3.12294578407668</v>
       </c>
       <c r="C463" s="2" t="n">
-        <v>-41.7652036328292</v>
+        <v>-41.7647259249018</v>
       </c>
       <c r="D463" s="2" t="n">
         <v>77</v>
@@ -19170,10 +19197,10 @@
         <v>1856</v>
       </c>
       <c r="H463" s="2" t="n">
+        <v>103</v>
+      </c>
+      <c r="I463" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="I463" s="2" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19181,10 +19208,10 @@
         <v>1857</v>
       </c>
       <c r="B464" s="2" t="n">
-        <v>-3.12254787337271</v>
+        <v>-3.1223398743864</v>
       </c>
       <c r="C464" s="2" t="n">
-        <v>-41.7644020536924</v>
+        <v>-41.7652036328292</v>
       </c>
       <c r="D464" s="2" t="n">
         <v>77</v>
@@ -19199,10 +19226,10 @@
         <v>1860</v>
       </c>
       <c r="H464" s="2" t="n">
-        <v>180</v>
+        <v>2</v>
       </c>
       <c r="I464" s="2" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19210,10 +19237,10 @@
         <v>1861</v>
       </c>
       <c r="B465" s="2" t="n">
-        <v>-3.1234002758931</v>
+        <v>-3.12254787337271</v>
       </c>
       <c r="C465" s="2" t="n">
-        <v>-41.7644470357224</v>
+        <v>-41.7644020536924</v>
       </c>
       <c r="D465" s="2" t="n">
         <v>77</v>
@@ -19228,7 +19255,7 @@
         <v>1864</v>
       </c>
       <c r="H465" s="2" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="I465" s="2" t="n">
         <v>2</v>
@@ -19239,10 +19266,10 @@
         <v>1865</v>
       </c>
       <c r="B466" s="2" t="n">
-        <v>-3.12288247964894</v>
+        <v>-3.1234002758931</v>
       </c>
       <c r="C466" s="2" t="n">
-        <v>-41.7635473934309</v>
+        <v>-41.7644470357224</v>
       </c>
       <c r="D466" s="2" t="n">
         <v>77</v>
@@ -19257,10 +19284,68 @@
         <v>1868</v>
       </c>
       <c r="H466" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="I466" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I466" s="2" t="n">
+    </row>
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A467" s="2" t="s">
+        <v>1869</v>
+      </c>
+      <c r="B467" s="2" t="n">
+        <v>-3.12288247955997</v>
+      </c>
+      <c r="C467" s="2" t="n">
+        <v>-41.7634574291974</v>
+      </c>
+      <c r="D467" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="E467" s="2" t="s">
+        <v>1870</v>
+      </c>
+      <c r="F467" s="2" t="s">
+        <v>1871</v>
+      </c>
+      <c r="G467" s="2" t="s">
+        <v>1872</v>
+      </c>
+      <c r="H467" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I467" s="2" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A468" s="2" t="s">
+        <v>1873</v>
+      </c>
+      <c r="B468" s="2" t="n">
+        <v>-3.12373676077234</v>
+      </c>
+      <c r="C468" s="2" t="n">
+        <v>-41.7651406020182</v>
+      </c>
+      <c r="D468" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="E468" s="2" t="s">
+        <v>1874</v>
+      </c>
+      <c r="F468" s="2" t="s">
+        <v>1875</v>
+      </c>
+      <c r="G468" s="2" t="s">
+        <v>1876</v>
+      </c>
+      <c r="H468" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I468" s="2" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="1048554" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>